<commit_message>
Small updates and presentation material
</commit_message>
<xml_diff>
--- a/01_Hardware/BoM.xlsx
+++ b/01_Hardware/BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/sachinumans_tudelft_nl/Documents/Documents/01a_Physical_Experiment/ActuatedPorousDisk_fabrication/01_Hardware/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/sachinumans_tudelft_nl/Documents/Documents/01_mainProject/Experimental/ActuatedPorousDisk_fabrication/01_Hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="436" documentId="8_{E9015A34-CF2A-4CF8-B73E-E4BD491994F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7A38F50-7C0D-4BC2-8A76-9A4051EE5DA6}"/>
+  <xr:revisionPtr revIDLastSave="437" documentId="8_{E9015A34-CF2A-4CF8-B73E-E4BD491994F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F1E2221-939E-4FE3-9BA5-B1D417235984}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{21B984F4-F71A-4ACE-8DA9-27D7BD98C737}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{21B984F4-F71A-4ACE-8DA9-27D7BD98C737}"/>
   </bookViews>
   <sheets>
     <sheet name="PorousDisk" sheetId="1" r:id="rId1"/>
@@ -444,10 +444,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -797,22 +793,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AECCCAA8-E429-414C-8D5A-69B27C1A67E9}">
   <dimension ref="A1:M25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" style="5" customWidth="1"/>
-    <col min="8" max="9" width="13.88671875" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" customWidth="1"/>
-    <col min="12" max="12" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" style="5" customWidth="1"/>
+    <col min="8" max="9" width="13.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="17.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -851,7 +847,7 @@
         <v>77.063355371900826</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>58</v>
       </c>
@@ -891,7 +887,7 @@
         <v>48.735537190082646</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -929,7 +925,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
@@ -964,7 +960,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -994,7 +990,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>62</v>
       </c>
@@ -1024,7 +1020,7 @@
         <v>0.35000000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>68</v>
       </c>
@@ -1060,7 +1056,7 @@
       </c>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>48</v>
       </c>
@@ -1095,7 +1091,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>47</v>
       </c>
@@ -1133,7 +1129,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>66</v>
       </c>
@@ -1168,7 +1164,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>70</v>
       </c>
@@ -1203,7 +1199,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>72</v>
       </c>
@@ -1236,7 +1232,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
@@ -1278,7 +1274,7 @@
         <v>2.6940495867768592</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1316,7 +1312,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
@@ -1354,7 +1350,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>29</v>
       </c>
@@ -1392,7 +1388,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1430,7 +1426,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>37</v>
       </c>
@@ -1472,7 +1468,7 @@
         <v>25.633768595041325</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1511,7 +1507,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>10</v>
       </c>
@@ -1550,7 +1546,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>13</v>
       </c>
@@ -1589,7 +1585,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1627,7 +1623,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>45</v>
       </c>
@@ -1662,7 +1658,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>34</v>
       </c>
@@ -1697,7 +1693,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
   </sheetData>

</xml_diff>